<commit_message>
Tham chiếu tới dự án LedOn
</commit_message>
<xml_diff>
--- a/Design.xlsx
+++ b/Design.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\FPGA\FPGA-DevKits\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A61376C-5E64-4E0B-818C-8497A448638F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ED6E567-1A9C-43C8-9B9D-3990714B7826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GPIO" sheetId="1" r:id="rId1"/>
-    <sheet name="Board" sheetId="3" r:id="rId2"/>
-    <sheet name="bits - hwh" sheetId="2" r:id="rId3"/>
+    <sheet name="laptop-board" sheetId="5" r:id="rId2"/>
+    <sheet name="Board" sheetId="3" r:id="rId3"/>
+    <sheet name="SNN_LIF" sheetId="4" r:id="rId4"/>
+    <sheet name="bits - hwh" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1900,6 +1902,321 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
+      <xdr:colOff>111610</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>896</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>249977</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>41366</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{361C278E-CF93-4834-9DDE-F67EC1CDFA5C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="1675" t="4935" r="2399" b="5018"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4988410" y="732416"/>
+          <a:ext cx="4405567" cy="2783670"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>68833</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>373381</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>111163</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A9D2F9E-1C76-27F9-A1C9-64921BA0621D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:clrChange>
+            <a:clrFrom>
+              <a:srgbClr val="FFFFFF"/>
+            </a:clrFrom>
+            <a:clrTo>
+              <a:srgbClr val="FFFFFF">
+                <a:alpha val="0"/>
+              </a:srgbClr>
+            </a:clrTo>
+          </a:clrChange>
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="609601" y="1166113"/>
+          <a:ext cx="2811780" cy="2054010"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>109560</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>115736</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>224118</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>54148</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="4" name="Ink 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9772BA97-024E-F4F2-6A54-454C37CB9485}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="3157560" y="2446560"/>
+            <a:ext cx="1943358" cy="297000"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="4" name="Ink 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9772BA97-024E-F4F2-6A54-454C37CB9485}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="3121559" y="2410560"/>
+              <a:ext cx="2015001" cy="368640"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>70980</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>76373</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>225462</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>51476</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="5" name="Ink 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CD1F919B-960E-C90C-FD52-150386E55EC3}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="3118980" y="1905173"/>
+            <a:ext cx="1983282" cy="706623"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="5" name="Ink 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CD1F919B-960E-C90C-FD52-150386E55EC3}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="3082979" y="1868795"/>
+              <a:ext cx="2054924" cy="779747"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>99956</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>43927</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1285160" cy="342786"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="TextBox 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1006CBFF-7D2B-858E-0245-0D4FAABE3257}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3757556" y="1506967"/>
+          <a:ext cx="1285160" cy="342786"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1600" b="1"/>
+            <a:t>192.168.2.99</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>9208</xdr:colOff>
       <xdr:row>41</xdr:row>
       <xdr:rowOff>172382</xdr:rowOff>
@@ -1989,8 +2306,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1712260" y="1048871"/>
-          <a:ext cx="7440706" cy="4661648"/>
+          <a:off x="1732431" y="1066800"/>
+          <a:ext cx="7528111" cy="4754881"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4103,7 +4420,1347 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>17931</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>51</xdr:col>
+      <xdr:colOff>9862</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>152401</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="36" name="Picture 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A0F0CDAC-E434-4F13-A7AD-BBBA6499D0B2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="1675" t="4935" r="2399" b="5018"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1732431" y="1066800"/>
+          <a:ext cx="7528111" cy="4754881"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="37" name="Speech Bubble: Rectangle 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DBDDA60A-3FF0-4E91-921E-4B1E3DFA22A2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3421380" y="6111240"/>
+          <a:ext cx="1524000" cy="815340"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 31353"/>
+            <a:gd name="adj2" fmla="val -143137"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>PROG</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US"/>
+            <a:t>Xóa cấu hình hiện tại của vùng FPGA và buộc nó phải nạp lại từ đầu.</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>180133</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>62948</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>46383</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>146767</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="38" name="Speech Bubble: Rectangle 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2DE5F7B4-610D-46E0-84F8-AE3139589DE2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5133133" y="6097988"/>
+          <a:ext cx="818750" cy="815339"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -39768"/>
+            <a:gd name="adj2" fmla="val -123081"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>SRST</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US"/>
+            <a:t>Khởi</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" baseline="0"/>
+            <a:t> động lại toàn bộ Dev Kit</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>99390</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>18883</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>26894</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>134470</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="39" name="Speech Bubble: Rectangle 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{604142C3-4DD2-4A0E-A9FB-99D996459F11}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3685272" y="4680530"/>
+          <a:ext cx="823975" cy="653469"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -6864"/>
+            <a:gd name="adj2" fmla="val -112696"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>SW</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>0</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>M20</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Reset</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>38430</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>66592</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>167640</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="41" name="Speech Bubble: Rectangle 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D56C32F7-51A8-4ED2-B333-001F7347BA2F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3718890" y="2809792"/>
+          <a:ext cx="1005510" cy="642068"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -36967"/>
+            <a:gd name="adj2" fmla="val 84731"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>R</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>G</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>B</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>0</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>N15</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>G17</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>L15</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>1Hz Clock</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>161365</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>73216</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="43" name="Speech Bubble: Rectangle 42">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A1C3CBDB-6D3E-4F10-87E5-D56BAFCAD9E2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6257365" y="4914157"/>
+          <a:ext cx="555811" cy="643961"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 36001"/>
+            <a:gd name="adj2" fmla="val -114609"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>BTN3</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>L</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>19</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" b="0"/>
+            <a:t>W=17</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>50327</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>64252</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>71717</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>170329</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="44" name="Speech Bubble: Rectangle 43">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{18661814-3002-4545-AAF1-319948BDB749}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6863503" y="4905193"/>
+          <a:ext cx="559273" cy="643960"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 17198"/>
+            <a:gd name="adj2" fmla="val -120307"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>BTN2</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>L20</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US"/>
+            <a:t>W=14</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>137893</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>73216</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>62752</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>170328</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="45" name="Speech Bubble: Rectangle 44">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BCAB971E-C6A5-454C-91E1-18C97C98BD3F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7488952" y="4914157"/>
+          <a:ext cx="642035" cy="634995"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 17198"/>
+            <a:gd name="adj2" fmla="val -120307"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>BTN1</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>D20</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US"/>
+            <a:t>W=20</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>45</xdr:col>
+      <xdr:colOff>126850</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>73217</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>49</xdr:col>
+      <xdr:colOff>35859</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="46" name="Speech Bubble: Rectangle 45">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BA3B77E4-2EF6-427A-A48E-4024BB4B9373}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8195085" y="4914158"/>
+          <a:ext cx="626186" cy="643960"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -22888"/>
+            <a:gd name="adj2" fmla="val -96641"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>BTN0</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>D19</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US"/>
+            <a:t>W=24</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>79513</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>106018</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>183197</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="47" name="Speech Bubble: Rectangle 46">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{70394968-A5B2-46B9-8763-C606243F6CCD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="841513" y="4678018"/>
+          <a:ext cx="865684" cy="442623"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 127427"/>
+            <a:gd name="adj2" fmla="val 13126"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>DC1 Power</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>7v ~ 15v</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>68180</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>120141</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>181803</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>14125</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="50" name="Speech Bubble: Rectangle 49">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6600D9C-FE63-403D-A7D9-D5A05297A00A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="830180" y="4143501"/>
+          <a:ext cx="875623" cy="442624"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 127427"/>
+            <a:gd name="adj2" fmla="val 13126"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Micro</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> USB</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2056</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>146003</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>105741</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>39986</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="52" name="Speech Bubble: Rectangle 51">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6F215293-B251-4C88-BFE9-DD2CA9D45EDE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1526056" y="5266643"/>
+          <a:ext cx="865685" cy="442623"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val 179953"/>
+            <a:gd name="adj2" fmla="val -166064"/>
+          </a:avLst>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FF0000"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Led</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t> đỏ </a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>báo nguồn</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1">
+            <a:solidFill>
+              <a:schemeClr val="bg1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>36</xdr:col>
+      <xdr:colOff>127303</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>174094</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>56</xdr:col>
+      <xdr:colOff>89989</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>40756</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="53" name="Picture 52" descr="Finger Touch Png, Transparent Png - kindpng">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A2D9E825-A43A-4180-A588-B61AEB958B8A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{BEBA8EAE-BF5A-486C-A8C5-ECC9F3942E4B}">
+              <a14:imgProps xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+                <a14:imgLayer r:embed="rId3">
+                  <a14:imgEffect>
+                    <a14:backgroundRemoval t="10000" b="90000" l="9302" r="90000">
+                      <a14:foregroundMark x1="9302" y1="88824" x2="9302" y2="88824"/>
+                    </a14:backgroundRemoval>
+                  </a14:imgEffect>
+                </a14:imgLayer>
+              </a14:imgProps>
+            </a:ext>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm rot="20506851">
+          <a:off x="6581891" y="1967035"/>
+          <a:ext cx="3548569" cy="2018192"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>106113</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>12804</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>53788</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>134470</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="59" name="Speech Bubble: Rectangle 58">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B7DF135-E33A-49FC-9235-8F033D00B679}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5484937" y="1985039"/>
+          <a:ext cx="1919910" cy="659549"/>
+        </a:xfrm>
+        <a:prstGeom prst="wedgeRectCallout">
+          <a:avLst>
+            <a:gd name="adj1" fmla="val -14410"/>
+            <a:gd name="adj2" fmla="val 39079"/>
+          </a:avLst>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:lnRef>
+        <a:fillRef idx="2">
+          <a:schemeClr val="accent4"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent4"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" b="1"/>
+            <a:t>SNN Leak Intergrate</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" b="1" baseline="0"/>
+            <a:t> and Fire</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="en-US"/>
+            <a:t>LEAK = 10</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US"/>
+            <a:t>THRESHOLD=100</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>152401</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>116542</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>89647</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>40770</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="60" name="Picture 59">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00A37EE8-A14F-45BB-433B-7F9815F7A183}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="500744" y="301599"/>
+          <a:ext cx="4291532" cy="2329971"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="bg1">
+              <a:lumMod val="65000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -4902,6 +6559,62 @@
     </inkml:brush>
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">1 1 24575,'10'1'0,"1"0"0,-1 1 0,0 0 0,0 0 0,0 1 0,0 1 0,0 0 0,-1 0 0,12 8 0,-4-3 0,-1 2 0,-1 0 0,0 0 0,17 18 0,-31-28 0,0 0 0,0 0 0,0 0 0,0 0 0,0 1 0,-1-1 0,1 0 0,0 0 0,-1 0 0,1 1 0,-1-1 0,1 0 0,-1 1 0,0-1 0,1 0 0,-1 1 0,0-1 0,0 0 0,0 1 0,0-1 0,0 0 0,0 1 0,0-1 0,-1 1 0,1-1 0,0 0 0,-1 0 0,1 1 0,-1-1 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,1 0 0,-3 2 0,-5 4 0,1 0 0,-2 0 0,1-1 0,-12 8 0,-14 11 0,22-13-455,0 1 0,-19 28 0,26-32-6371</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink13.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-10-21T05:52:56.278"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.2" units="cm"/>
+      <inkml:brushProperty name="height" value="0.2" units="cm"/>
+      <inkml:brushProperty name="color" value="#E71224"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">26 824 24575,'-25'-52'0,"25"49"0,0 0 0,-1 1 0,2-1 0,-1 1 0,0-1 0,1 1 0,0-1 0,-1 1 0,1 0 0,1-1 0,-1 1 0,0 0 0,1-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 1 0,-1-1 0,1 0 0,0 1 0,0 0 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,4 0 0,13-3 0,-1 1 0,1 0 0,0 1 0,29 0 0,8-2 0,-25 0 0,-12 3 0,1-2 0,-1 0 0,1 0 0,-1-1 0,-1-1 0,1-1 0,30-12 0,-33 11 0,0 0 0,1 1 0,0 1 0,0 0 0,1 0 0,-1 2 0,2 0 0,-1 0 0,0 1 0,1 1 0,-1 0 0,29 2 0,-36-1 0,1 0 0,0-1 0,-1-1 0,1 1 0,-1-2 0,1 1 0,-1-1 0,16-6 0,6-3 0,46-24 0,-49 21 0,0 1 0,34-10 0,-29 13 0,0 1 0,1 1 0,0 1 0,56-6 0,-57 9 0,65-15 0,-15 3 0,35-5 0,197-54 0,-254 59 0,1 3 0,96-13 0,-87 16 0,112-27 0,91-26 0,-32 9 0,-196 42 0,0 2 0,1 1 0,0 2 0,1 2 0,0 2 0,80-1 0,906 8 0,-592-4 0,-419 2 0,-1 1 0,45 8 0,-42-6 0,-1 0 0,33 1 0,108-5-1365</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink14.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-10-21T05:53:05.186"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.2" units="cm"/>
+      <inkml:brushProperty name="height" value="0.2" units="cm"/>
+      <inkml:brushProperty name="color" value="#00A0D7"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">5508 1 24575,'0'1'0,"-1"0"0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,0 0 0,-1-1 0,1 1 0,0 0 0,-1-1 0,1 1 0,-1 0 0,1-1 0,-1 0 0,1 1 0,-1-1 0,1 1 0,-1-1 0,0 0 0,1 0 0,-4 0 0,-52 5 0,51-5 0,-70 2 0,36-1 0,0 1 0,-68 9 0,-50 6 0,66-8 0,57-6 0,-294 29 0,304-29 0,0 1 0,0 1 0,1 0 0,0 2 0,0-1 0,-23 11 0,17-6 0,-1-2 0,-1 0 0,-36 6 0,-99 14 0,59-9 0,-173 16 0,242-31 0,0 1 0,1 1 0,0 2 0,-50 15 0,41-10 0,-3 0 0,-252 74 0,34 9 0,47-17 0,49-23 0,-135 49 0,150-45 0,77-33 0,1 3 0,2 3 0,-100 58 0,144-74 0,0-1 0,-2-2 0,-61 22 0,52-21 0,1 1 0,-40 22 0,32-11 0,1 1 0,2 1 0,2 2 0,-60 54 0,68-53 0,-68 46 0,78-59 0,-113 75 0,102-67 0,-42 39 0,-14 11 0,75-65 0,-1-1 0,0 0 0,-25 9 0,-38 21 0,32-14-1365</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -5768,6 +7481,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9003CB8E-8A37-48F8-AF17-EF837193EE59}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{968AC48A-2378-4E91-8413-C6C5E438A215}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="2.77734375" defaultRowHeight="14.4"/>
@@ -5777,7 +7500,18 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78C856A6-90BD-40C6-A676-6048191FCA79}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="2.5546875" defaultRowHeight="14.4"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C38D68DB-870D-4233-B871-A8BC2088FA29}">
   <dimension ref="B2:AL19"/>
   <sheetFormatPr defaultColWidth="2.77734375" defaultRowHeight="14.4"/>

</xml_diff>